<commit_message>
Fix NaN encoding in JSON exports and workflow copy steps
</commit_message>
<xml_diff>
--- a/data/market/market_model.xlsx
+++ b/data/market/market_model.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="105">
   <si>
     <t>key</t>
   </si>
@@ -54,9 +54,6 @@
     <t>firms</t>
   </si>
   <si>
-    <t>60000</t>
-  </si>
-  <si>
     <t>SOURCED</t>
   </si>
   <si>
@@ -72,9 +69,6 @@
     <t>firms_mid</t>
   </si>
   <si>
-    <t>300000</t>
-  </si>
-  <si>
     <t>ASSUMPTION</t>
   </si>
   <si>
@@ -87,18 +81,12 @@
     <t>share</t>
   </si>
   <si>
-    <t>0.70</t>
-  </si>
-  <si>
     <t>Large enterprises are more likely to have a modern data platform</t>
   </si>
   <si>
     <t>adoption_mid</t>
   </si>
   <si>
-    <t>0.35</t>
-  </si>
-  <si>
     <t>Mid market adoption is growing but trails large enterprise</t>
   </si>
   <si>
@@ -108,18 +96,12 @@
     <t>USD</t>
   </si>
   <si>
-    <t>2000000</t>
-  </si>
-  <si>
     <t>Average annual platform spend for large enterprise</t>
   </si>
   <si>
     <t>spend_mid</t>
   </si>
   <si>
-    <t>200000</t>
-  </si>
-  <si>
     <t>Average annual platform spend for mid market</t>
   </si>
   <si>
@@ -132,27 +114,18 @@
     <t>share_wh</t>
   </si>
   <si>
-    <t>0.40</t>
-  </si>
-  <si>
     <t>SQL analytics and BI is the core warehouse use case</t>
   </si>
   <si>
     <t>share_stream</t>
   </si>
   <si>
-    <t>0.15</t>
-  </si>
-  <si>
     <t>Streaming is growing but still smaller share of spend</t>
   </si>
   <si>
     <t>share_ai</t>
   </si>
   <si>
-    <t>0.20</t>
-  </si>
-  <si>
     <t>AI/ML preparation spend is increasing rapidly</t>
   </si>
   <si>
@@ -165,9 +138,6 @@
     <t>deploy_public</t>
   </si>
   <si>
-    <t>0.75</t>
-  </si>
-  <si>
     <t>Public cloud is the dominant deployment mode</t>
   </si>
   <si>
@@ -180,9 +150,6 @@
     <t>deploy_hybrid</t>
   </si>
   <si>
-    <t>0.25</t>
-  </si>
-  <si>
     <t>Hybrid spans both</t>
   </si>
   <si>
@@ -192,9 +159,6 @@
     <t>rate</t>
   </si>
   <si>
-    <t>0.16</t>
-  </si>
-  <si>
     <t>Steady growth for data engineering</t>
   </si>
   <si>
@@ -207,18 +171,12 @@
     <t>cagr_stream</t>
   </si>
   <si>
-    <t>0.30</t>
-  </si>
-  <si>
     <t>High growth in real-time use cases</t>
   </si>
   <si>
     <t>cagr_ai</t>
   </si>
   <si>
-    <t>0.45</t>
-  </si>
-  <si>
     <t>Fastest growing segment due to GenAI</t>
   </si>
   <si>
@@ -231,16 +189,10 @@
     <t>cagr_deploy_public</t>
   </si>
   <si>
-    <t>0.26</t>
-  </si>
-  <si>
     <t>Public cloud growing faster than on-prem</t>
   </si>
   <si>
     <t>cagr_deploy_private</t>
-  </si>
-  <si>
-    <t>0.00</t>
   </si>
   <si>
     <t>On-prem is shrinking slowly</t>
@@ -780,25 +732,25 @@
       <c r="E2">
         <v>50000</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2">
+        <v>60000</v>
+      </c>
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3">
         <v>250000</v>
@@ -812,25 +764,25 @@
       <c r="E3">
         <v>250000</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3">
+        <v>300000</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
         <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B4">
         <v>0.6</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D4">
         <v>0.5</v>
@@ -838,25 +790,25 @@
       <c r="E4">
         <v>0.6</v>
       </c>
-      <c r="F4" t="s">
-        <v>23</v>
+      <c r="F4">
+        <v>0.7</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>0.25</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D5">
         <v>0.15</v>
@@ -864,25 +816,25 @@
       <c r="E5">
         <v>0.25</v>
       </c>
-      <c r="F5" t="s">
-        <v>26</v>
+      <c r="F5">
+        <v>0.35</v>
       </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>1500000</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D6">
         <v>1000000</v>
@@ -890,25 +842,25 @@
       <c r="E6">
         <v>1500000</v>
       </c>
-      <c r="F6" t="s">
-        <v>30</v>
+      <c r="F6">
+        <v>2000000</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J6" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>150000</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D7">
         <v>100000</v>
@@ -916,25 +868,25 @@
       <c r="E7">
         <v>150000</v>
       </c>
-      <c r="F7" t="s">
-        <v>33</v>
+      <c r="F7">
+        <v>200000</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J7" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B8">
         <v>0.3</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D8">
         <v>0.25</v>
@@ -942,25 +894,25 @@
       <c r="E8">
         <v>0.3</v>
       </c>
-      <c r="F8" t="s">
-        <v>26</v>
+      <c r="F8">
+        <v>0.35</v>
       </c>
       <c r="G8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J8" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>0.35</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D9">
         <v>0.3</v>
@@ -968,25 +920,25 @@
       <c r="E9">
         <v>0.35</v>
       </c>
-      <c r="F9" t="s">
-        <v>38</v>
+      <c r="F9">
+        <v>0.4</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J9" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B10">
         <v>0.1</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D10">
         <v>0.05</v>
@@ -994,25 +946,25 @@
       <c r="E10">
         <v>0.1</v>
       </c>
-      <c r="F10" t="s">
-        <v>41</v>
+      <c r="F10">
+        <v>0.15</v>
       </c>
       <c r="G10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J10" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>0.15</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D11">
         <v>0.1</v>
@@ -1020,25 +972,25 @@
       <c r="E11">
         <v>0.15</v>
       </c>
-      <c r="F11" t="s">
-        <v>44</v>
+      <c r="F11">
+        <v>0.2</v>
       </c>
       <c r="G11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J11" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B12">
         <v>0.1</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D12">
         <v>0.05</v>
@@ -1046,25 +998,25 @@
       <c r="E12">
         <v>0.1</v>
       </c>
-      <c r="F12" t="s">
-        <v>41</v>
+      <c r="F12">
+        <v>0.15</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J12" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B13">
         <v>0.65</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D13">
         <v>0.55</v>
@@ -1072,25 +1024,25 @@
       <c r="E13">
         <v>0.65</v>
       </c>
-      <c r="F13" t="s">
-        <v>49</v>
+      <c r="F13">
+        <v>0.75</v>
       </c>
       <c r="G13" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J13" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="B14">
         <v>0.15</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D14">
         <v>0.1</v>
@@ -1098,25 +1050,25 @@
       <c r="E14">
         <v>0.15</v>
       </c>
-      <c r="F14" t="s">
-        <v>44</v>
+      <c r="F14">
+        <v>0.2</v>
       </c>
       <c r="G14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J14" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="B15">
         <v>0.2</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D15">
         <v>0.15</v>
@@ -1124,25 +1076,25 @@
       <c r="E15">
         <v>0.2</v>
       </c>
-      <c r="F15" t="s">
-        <v>54</v>
+      <c r="F15">
+        <v>0.25</v>
       </c>
       <c r="G15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J15" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>0.12</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D16">
         <v>0.08</v>
@@ -1150,25 +1102,25 @@
       <c r="E16">
         <v>0.12</v>
       </c>
-      <c r="F16" t="s">
-        <v>58</v>
+      <c r="F16">
+        <v>0.16</v>
       </c>
       <c r="G16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J16" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B17">
         <v>0.1</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D17">
         <v>0.05</v>
@@ -1176,25 +1128,25 @@
       <c r="E17">
         <v>0.1</v>
       </c>
-      <c r="F17" t="s">
-        <v>41</v>
+      <c r="F17">
+        <v>0.15</v>
       </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J17" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="B18">
         <v>0.25</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D18">
         <v>0.2</v>
@@ -1202,25 +1154,25 @@
       <c r="E18">
         <v>0.25</v>
       </c>
-      <c r="F18" t="s">
-        <v>63</v>
+      <c r="F18">
+        <v>0.3</v>
       </c>
       <c r="G18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J18" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="B19">
         <v>0.35</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D19">
         <v>0.25</v>
@@ -1228,25 +1180,25 @@
       <c r="E19">
         <v>0.35</v>
       </c>
-      <c r="F19" t="s">
-        <v>66</v>
+      <c r="F19">
+        <v>0.45</v>
       </c>
       <c r="G19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J19" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>0.2</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D20">
         <v>0.15</v>
@@ -1254,25 +1206,25 @@
       <c r="E20">
         <v>0.2</v>
       </c>
-      <c r="F20" t="s">
-        <v>54</v>
+      <c r="F20">
+        <v>0.25</v>
       </c>
       <c r="G20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J20" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B21">
         <v>0.22</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D21">
         <v>0.18</v>
@@ -1280,25 +1232,25 @@
       <c r="E21">
         <v>0.22</v>
       </c>
-      <c r="F21" t="s">
-        <v>71</v>
+      <c r="F21">
+        <v>0.26</v>
       </c>
       <c r="G21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J21" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B22">
         <v>-0.05</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D22">
         <v>-0.1</v>
@@ -1306,25 +1258,25 @@
       <c r="E22">
         <v>-0.05</v>
       </c>
-      <c r="F22" t="s">
-        <v>74</v>
+      <c r="F22">
+        <v>0</v>
       </c>
       <c r="G22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J22" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B23">
         <v>0.15</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D23">
         <v>0.1</v>
@@ -1332,84 +1284,84 @@
       <c r="E23">
         <v>0.15</v>
       </c>
-      <c r="F23" t="s">
-        <v>44</v>
+      <c r="F23">
+        <v>0.2</v>
       </c>
       <c r="G23" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J23" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B24">
         <v>3500000000</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
-      </c>
-      <c r="F24" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="H24" t="s">
-        <v>15</v>
+        <v>25</v>
+      </c>
+      <c r="G24" t="s">
+        <v>12</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="I24" t="s">
-        <v>80</v>
+        <v>14</v>
+      </c>
+      <c r="J24" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="B25">
         <v>2400000000</v>
       </c>
       <c r="C25" t="s">
-        <v>29</v>
-      </c>
-      <c r="F25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H25" t="s">
-        <v>15</v>
+        <v>25</v>
+      </c>
+      <c r="G25" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="I25" t="s">
-        <v>83</v>
+        <v>14</v>
+      </c>
+      <c r="J25" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="B26">
         <v>15000000000</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
-      </c>
-      <c r="F26" t="s">
-        <v>19</v>
-      </c>
-      <c r="I26" t="s">
-        <v>85</v>
+        <v>25</v>
+      </c>
+      <c r="G26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1"/>
-    <hyperlink ref="G24" r:id="rId2"/>
-    <hyperlink ref="G25" r:id="rId3"/>
+    <hyperlink ref="H24" r:id="rId2"/>
+    <hyperlink ref="H25" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1422,51 +1374,51 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="B1" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="C1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E1" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="F1" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="G1" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="H1" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="I1" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="J1" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="K1" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E2" s="2">
         <v>3510000000</v>
@@ -1493,16 +1445,16 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E3" s="2">
         <v>2632500000</v>
@@ -1529,16 +1481,16 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E4" s="2">
         <v>1930500000</v>
@@ -1565,16 +1517,16 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E5" s="2">
         <v>702000000</v>
@@ -1601,16 +1553,16 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E6" s="2">
         <v>731250000</v>
@@ -1637,16 +1589,16 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D7" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E7" s="2">
         <v>548437500</v>
@@ -1673,16 +1625,16 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E8" s="2">
         <v>402187500</v>
@@ -1709,16 +1661,16 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E9" s="2">
         <v>146250000</v>
@@ -1745,16 +1697,16 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E10" s="2">
         <v>810000000</v>
@@ -1781,16 +1733,16 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E11" s="2">
         <v>607500000</v>
@@ -1817,16 +1769,16 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D12" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E12" s="2">
         <v>445500000</v>
@@ -1853,16 +1805,16 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E13" s="2">
         <v>162000000</v>
@@ -1889,16 +1841,16 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E14" s="2">
         <v>168750000</v>
@@ -1925,16 +1877,16 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D15" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E15" s="2">
         <v>126562500</v>
@@ -1961,16 +1913,16 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E16" s="2">
         <v>92812500</v>
@@ -1997,16 +1949,16 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E17" s="2">
         <v>33750000</v>
@@ -2033,16 +1985,16 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B18" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D18" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E18" s="2">
         <v>1080000000</v>
@@ -2069,16 +2021,16 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D19" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E19" s="2">
         <v>810000000</v>
@@ -2105,16 +2057,16 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E20" s="2">
         <v>594000000</v>
@@ -2141,16 +2093,16 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D21" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E21" s="2">
         <v>216000000</v>
@@ -2177,16 +2129,16 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B22" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E22" s="2">
         <v>225000000</v>
@@ -2213,16 +2165,16 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E23" s="2">
         <v>168750000</v>
@@ -2249,16 +2201,16 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D24" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E24" s="2">
         <v>123750000</v>
@@ -2285,16 +2237,16 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D25" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E25" s="2">
         <v>45000000</v>
@@ -2321,16 +2273,16 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C26" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E26" s="2">
         <v>4095000000</v>
@@ -2357,16 +2309,16 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B27" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E27" s="2">
         <v>3071250000</v>
@@ -2393,16 +2345,16 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C28" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D28" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E28" s="2">
         <v>2252250000</v>
@@ -2429,16 +2381,16 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B29" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C29" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E29" s="2">
         <v>819000000</v>
@@ -2465,16 +2417,16 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B30" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D30" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E30" s="2">
         <v>853125000</v>
@@ -2501,16 +2453,16 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B31" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C31" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E31" s="2">
         <v>639843750</v>
@@ -2537,16 +2489,16 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B32" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C32" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D32" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E32" s="2">
         <v>469218750</v>
@@ -2573,16 +2525,16 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B33" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D33" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E33" s="2">
         <v>170625000</v>
@@ -2609,16 +2561,16 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B34" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D34" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E34" s="2">
         <v>945000000</v>
@@ -2645,16 +2597,16 @@
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D35" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E35" s="2">
         <v>708750000</v>
@@ -2681,16 +2633,16 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C36" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D36" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E36" s="2">
         <v>519750000</v>
@@ -2717,16 +2669,16 @@
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B37" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C37" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D37" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E37" s="2">
         <v>189000000</v>
@@ -2753,16 +2705,16 @@
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C38" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D38" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E38" s="2">
         <v>196875000</v>
@@ -2789,16 +2741,16 @@
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B39" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C39" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D39" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E39" s="2">
         <v>147656250</v>
@@ -2825,16 +2777,16 @@
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B40" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C40" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E40" s="2">
         <v>108281250</v>
@@ -2861,16 +2813,16 @@
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B41" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C41" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D41" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E41" s="2">
         <v>39375000</v>
@@ -2897,16 +2849,16 @@
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B42" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D42" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E42" s="2">
         <v>1260000000</v>
@@ -2933,16 +2885,16 @@
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D43" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E43" s="2">
         <v>945000000</v>
@@ -2969,16 +2921,16 @@
     </row>
     <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B44" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D44" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E44" s="2">
         <v>693000000</v>
@@ -3005,16 +2957,16 @@
     </row>
     <row r="45" spans="1:11">
       <c r="A45" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B45" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C45" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D45" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E45" s="2">
         <v>252000000</v>
@@ -3041,16 +2993,16 @@
     </row>
     <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D46" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E46" s="2">
         <v>262500000</v>
@@ -3077,16 +3029,16 @@
     </row>
     <row r="47" spans="1:11">
       <c r="A47" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D47" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E47" s="2">
         <v>196875000</v>
@@ -3113,16 +3065,16 @@
     </row>
     <row r="48" spans="1:11">
       <c r="A48" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C48" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D48" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E48" s="2">
         <v>144375000</v>
@@ -3149,16 +3101,16 @@
     </row>
     <row r="49" spans="1:11">
       <c r="A49" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D49" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E49" s="2">
         <v>52500000</v>
@@ -3185,16 +3137,16 @@
     </row>
     <row r="50" spans="1:11">
       <c r="A50" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C50" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D50" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E50" s="2">
         <v>1170000000</v>
@@ -3221,16 +3173,16 @@
     </row>
     <row r="51" spans="1:11">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B51" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D51" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E51" s="2">
         <v>877500000</v>
@@ -3257,16 +3209,16 @@
     </row>
     <row r="52" spans="1:11">
       <c r="A52" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B52" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C52" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D52" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E52" s="2">
         <v>643500000</v>
@@ -3293,16 +3245,16 @@
     </row>
     <row r="53" spans="1:11">
       <c r="A53" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C53" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E53" s="2">
         <v>234000000</v>
@@ -3329,16 +3281,16 @@
     </row>
     <row r="54" spans="1:11">
       <c r="A54" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B54" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C54" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D54" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E54" s="2">
         <v>243750000</v>
@@ -3365,16 +3317,16 @@
     </row>
     <row r="55" spans="1:11">
       <c r="A55" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B55" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C55" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D55" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E55" s="2">
         <v>182812500</v>
@@ -3401,16 +3353,16 @@
     </row>
     <row r="56" spans="1:11">
       <c r="A56" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B56" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C56" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D56" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E56" s="2">
         <v>134062500</v>
@@ -3437,16 +3389,16 @@
     </row>
     <row r="57" spans="1:11">
       <c r="A57" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C57" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D57" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E57" s="2">
         <v>48750000</v>
@@ -3473,16 +3425,16 @@
     </row>
     <row r="58" spans="1:11">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B58" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C58" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E58" s="2">
         <v>270000000</v>
@@ -3509,16 +3461,16 @@
     </row>
     <row r="59" spans="1:11">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B59" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C59" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D59" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E59" s="2">
         <v>202500000</v>
@@ -3545,16 +3497,16 @@
     </row>
     <row r="60" spans="1:11">
       <c r="A60" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B60" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C60" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E60" s="2">
         <v>148500000</v>
@@ -3581,16 +3533,16 @@
     </row>
     <row r="61" spans="1:11">
       <c r="A61" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B61" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C61" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D61" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E61" s="2">
         <v>54000000</v>
@@ -3617,16 +3569,16 @@
     </row>
     <row r="62" spans="1:11">
       <c r="A62" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B62" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C62" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D62" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E62" s="2">
         <v>56250000</v>
@@ -3653,16 +3605,16 @@
     </row>
     <row r="63" spans="1:11">
       <c r="A63" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B63" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C63" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D63" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E63" s="2">
         <v>42187500</v>
@@ -3689,16 +3641,16 @@
     </row>
     <row r="64" spans="1:11">
       <c r="A64" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B64" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C64" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D64" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E64" s="2">
         <v>30937500</v>
@@ -3725,16 +3677,16 @@
     </row>
     <row r="65" spans="1:11">
       <c r="A65" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B65" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C65" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D65" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E65" s="2">
         <v>11250000</v>
@@ -3761,16 +3713,16 @@
     </row>
     <row r="66" spans="1:11">
       <c r="A66" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B66" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C66" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D66" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E66" s="2">
         <v>360000000</v>
@@ -3797,16 +3749,16 @@
     </row>
     <row r="67" spans="1:11">
       <c r="A67" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B67" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C67" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D67" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E67" s="2">
         <v>270000000</v>
@@ -3833,16 +3785,16 @@
     </row>
     <row r="68" spans="1:11">
       <c r="A68" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B68" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C68" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D68" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E68" s="2">
         <v>198000000</v>
@@ -3869,16 +3821,16 @@
     </row>
     <row r="69" spans="1:11">
       <c r="A69" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B69" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C69" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D69" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E69" s="2">
         <v>72000000</v>
@@ -3905,16 +3857,16 @@
     </row>
     <row r="70" spans="1:11">
       <c r="A70" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B70" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D70" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E70" s="2">
         <v>75000000</v>
@@ -3941,16 +3893,16 @@
     </row>
     <row r="71" spans="1:11">
       <c r="A71" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B71" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C71" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E71" s="2">
         <v>56250000</v>
@@ -3977,16 +3929,16 @@
     </row>
     <row r="72" spans="1:11">
       <c r="A72" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B72" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C72" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D72" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E72" s="2">
         <v>41250000</v>
@@ -4013,16 +3965,16 @@
     </row>
     <row r="73" spans="1:11">
       <c r="A73" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B73" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C73" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E73" s="2">
         <v>15000000</v>
@@ -4049,16 +4001,16 @@
     </row>
     <row r="74" spans="1:11">
       <c r="A74" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B74" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C74" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D74" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E74" s="2">
         <v>1755000000</v>
@@ -4085,16 +4037,16 @@
     </row>
     <row r="75" spans="1:11">
       <c r="A75" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B75" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C75" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D75" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E75" s="2">
         <v>1316250000</v>
@@ -4121,16 +4073,16 @@
     </row>
     <row r="76" spans="1:11">
       <c r="A76" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B76" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C76" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D76" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E76" s="2">
         <v>965250000</v>
@@ -4157,16 +4109,16 @@
     </row>
     <row r="77" spans="1:11">
       <c r="A77" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B77" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C77" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D77" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E77" s="2">
         <v>351000000</v>
@@ -4193,16 +4145,16 @@
     </row>
     <row r="78" spans="1:11">
       <c r="A78" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B78" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C78" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D78" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E78" s="2">
         <v>365625000</v>
@@ -4229,16 +4181,16 @@
     </row>
     <row r="79" spans="1:11">
       <c r="A79" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B79" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C79" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D79" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E79" s="2">
         <v>274218750</v>
@@ -4265,16 +4217,16 @@
     </row>
     <row r="80" spans="1:11">
       <c r="A80" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B80" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C80" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D80" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E80" s="2">
         <v>201093750</v>
@@ -4301,16 +4253,16 @@
     </row>
     <row r="81" spans="1:11">
       <c r="A81" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B81" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C81" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D81" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E81" s="2">
         <v>73125000</v>
@@ -4337,16 +4289,16 @@
     </row>
     <row r="82" spans="1:11">
       <c r="A82" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B82" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C82" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D82" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E82" s="2">
         <v>405000000</v>
@@ -4373,16 +4325,16 @@
     </row>
     <row r="83" spans="1:11">
       <c r="A83" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B83" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C83" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D83" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E83" s="2">
         <v>303750000</v>
@@ -4409,16 +4361,16 @@
     </row>
     <row r="84" spans="1:11">
       <c r="A84" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B84" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C84" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D84" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E84" s="2">
         <v>222750000</v>
@@ -4445,16 +4397,16 @@
     </row>
     <row r="85" spans="1:11">
       <c r="A85" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B85" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C85" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D85" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E85" s="2">
         <v>81000000</v>
@@ -4481,16 +4433,16 @@
     </row>
     <row r="86" spans="1:11">
       <c r="A86" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B86" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C86" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D86" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E86" s="2">
         <v>84375000</v>
@@ -4517,16 +4469,16 @@
     </row>
     <row r="87" spans="1:11">
       <c r="A87" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B87" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C87" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D87" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E87" s="2">
         <v>63281250</v>
@@ -4553,16 +4505,16 @@
     </row>
     <row r="88" spans="1:11">
       <c r="A88" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B88" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C88" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D88" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E88" s="2">
         <v>46406250</v>
@@ -4589,16 +4541,16 @@
     </row>
     <row r="89" spans="1:11">
       <c r="A89" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B89" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C89" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D89" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E89" s="2">
         <v>16875000</v>
@@ -4625,16 +4577,16 @@
     </row>
     <row r="90" spans="1:11">
       <c r="A90" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B90" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C90" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D90" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E90" s="2">
         <v>540000000</v>
@@ -4661,16 +4613,16 @@
     </row>
     <row r="91" spans="1:11">
       <c r="A91" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C91" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D91" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E91" s="2">
         <v>405000000</v>
@@ -4697,16 +4649,16 @@
     </row>
     <row r="92" spans="1:11">
       <c r="A92" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C92" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D92" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E92" s="2">
         <v>297000000</v>
@@ -4733,16 +4685,16 @@
     </row>
     <row r="93" spans="1:11">
       <c r="A93" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B93" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C93" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D93" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E93" s="2">
         <v>108000000</v>
@@ -4769,16 +4721,16 @@
     </row>
     <row r="94" spans="1:11">
       <c r="A94" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C94" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D94" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E94" s="2">
         <v>112500000</v>
@@ -4805,16 +4757,16 @@
     </row>
     <row r="95" spans="1:11">
       <c r="A95" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B95" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C95" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D95" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E95" s="2">
         <v>84375000</v>
@@ -4841,16 +4793,16 @@
     </row>
     <row r="96" spans="1:11">
       <c r="A96" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B96" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C96" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D96" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E96" s="2">
         <v>61875000</v>
@@ -4877,16 +4829,16 @@
     </row>
     <row r="97" spans="1:11">
       <c r="A97" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B97" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C97" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D97" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E97" s="2">
         <v>22500000</v>
@@ -4913,16 +4865,16 @@
     </row>
     <row r="98" spans="1:11">
       <c r="A98" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B98" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C98" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D98" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E98" s="2">
         <v>1170000000</v>
@@ -4949,16 +4901,16 @@
     </row>
     <row r="99" spans="1:11">
       <c r="A99" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B99" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C99" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D99" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E99" s="2">
         <v>877500000</v>
@@ -4985,16 +4937,16 @@
     </row>
     <row r="100" spans="1:11">
       <c r="A100" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B100" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C100" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D100" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E100" s="2">
         <v>643500000</v>
@@ -5021,16 +4973,16 @@
     </row>
     <row r="101" spans="1:11">
       <c r="A101" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B101" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C101" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D101" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E101" s="2">
         <v>234000000</v>
@@ -5057,16 +5009,16 @@
     </row>
     <row r="102" spans="1:11">
       <c r="A102" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B102" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C102" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D102" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E102" s="2">
         <v>243750000</v>
@@ -5093,16 +5045,16 @@
     </row>
     <row r="103" spans="1:11">
       <c r="A103" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B103" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C103" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D103" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E103" s="2">
         <v>182812500</v>
@@ -5129,16 +5081,16 @@
     </row>
     <row r="104" spans="1:11">
       <c r="A104" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B104" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C104" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D104" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E104" s="2">
         <v>134062500</v>
@@ -5165,16 +5117,16 @@
     </row>
     <row r="105" spans="1:11">
       <c r="A105" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B105" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="C105" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D105" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E105" s="2">
         <v>48750000</v>
@@ -5201,16 +5153,16 @@
     </row>
     <row r="106" spans="1:11">
       <c r="A106" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B106" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C106" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D106" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E106" s="2">
         <v>270000000</v>
@@ -5237,16 +5189,16 @@
     </row>
     <row r="107" spans="1:11">
       <c r="A107" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B107" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C107" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D107" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E107" s="2">
         <v>202500000</v>
@@ -5273,16 +5225,16 @@
     </row>
     <row r="108" spans="1:11">
       <c r="A108" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B108" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C108" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D108" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E108" s="2">
         <v>148500000</v>
@@ -5309,16 +5261,16 @@
     </row>
     <row r="109" spans="1:11">
       <c r="A109" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B109" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C109" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D109" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E109" s="2">
         <v>54000000</v>
@@ -5345,16 +5297,16 @@
     </row>
     <row r="110" spans="1:11">
       <c r="A110" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B110" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C110" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D110" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E110" s="2">
         <v>56250000</v>
@@ -5381,16 +5333,16 @@
     </row>
     <row r="111" spans="1:11">
       <c r="A111" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B111" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C111" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D111" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E111" s="2">
         <v>42187500</v>
@@ -5417,16 +5369,16 @@
     </row>
     <row r="112" spans="1:11">
       <c r="A112" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B112" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C112" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D112" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E112" s="2">
         <v>30937500</v>
@@ -5453,16 +5405,16 @@
     </row>
     <row r="113" spans="1:11">
       <c r="A113" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B113" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C113" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D113" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E113" s="2">
         <v>11250000</v>
@@ -5489,16 +5441,16 @@
     </row>
     <row r="114" spans="1:11">
       <c r="A114" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B114" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C114" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D114" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E114" s="2">
         <v>360000000</v>
@@ -5525,16 +5477,16 @@
     </row>
     <row r="115" spans="1:11">
       <c r="A115" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B115" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C115" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D115" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E115" s="2">
         <v>270000000</v>
@@ -5561,16 +5513,16 @@
     </row>
     <row r="116" spans="1:11">
       <c r="A116" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B116" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C116" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D116" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E116" s="2">
         <v>198000000</v>
@@ -5597,16 +5549,16 @@
     </row>
     <row r="117" spans="1:11">
       <c r="A117" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B117" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C117" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D117" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E117" s="2">
         <v>72000000</v>
@@ -5633,16 +5585,16 @@
     </row>
     <row r="118" spans="1:11">
       <c r="A118" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B118" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C118" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D118" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E118" s="2">
         <v>75000000</v>
@@ -5669,16 +5621,16 @@
     </row>
     <row r="119" spans="1:11">
       <c r="A119" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B119" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C119" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D119" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E119" s="2">
         <v>56250000</v>
@@ -5705,16 +5657,16 @@
     </row>
     <row r="120" spans="1:11">
       <c r="A120" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B120" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C120" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D120" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E120" s="2">
         <v>41250000</v>
@@ -5741,16 +5693,16 @@
     </row>
     <row r="121" spans="1:11">
       <c r="A121" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B121" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C121" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D121" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E121" s="2">
         <v>15000000</v>
@@ -5777,7 +5729,7 @@
     </row>
     <row r="122" spans="1:11">
       <c r="D122" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="E122" s="2">
         <f>SUM(E2:E121)</f>
@@ -5816,52 +5768,51 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="B1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="C1" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B2" s="2">
         <v>3500000000</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>79</v>
+      <c r="C2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="B3" s="2">
         <v>2400000000</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>82</v>
+      <c r="C3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="B4" s="2">
         <v>15000000000</v>
       </c>
-      <c r="C4" t="e">
-        <f>#NUM!</f>
-        <v>#NUM!</v>
+      <c r="C4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="B5" s="2">
         <f>SUM(B2:B4)</f>
@@ -5870,7 +5821,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="B6" s="2">
         <f>Segments!E122</f>
@@ -5879,7 +5830,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="B7" s="2">
         <f>B6-B5</f>
@@ -5887,10 +5838,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1"/>
-    <hyperlink ref="C3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>